<commit_message>
chore(finance): refresh cfo + powerbi — 2026-07-07 (loop iteration 1)
/finance-refresh via the 6-hour loop. First iteration with LIVE QuickBooks.

Source    Status   Detail                                    Checks
cfo       OK       LIVE QB pull — P&L FY24/FY25/YTD +        7/7
                   verified months May+Jun 2026.
                   YTD rev $30.24M (was $19.38M @ May 7),
                   GP $9.95M (GM 32.9%), net $4.54M.
                   Year-end forecast: rev $51.84M, net $7.79M.
                   Cash flow retained at 2026-05-07 vintage
                   (cash_flow tool needs approval; P&L tool
                   was allowlisted). Benchmark retained.
powerbi   OK       rebuilt + promoted, as-of 2026-06-17;     5/5
                   validator independently green
knowify   SKIPPED  KNOWIFY_USERNAME/PASSWORD not set         —

June 2026 was the strongest month on record: $5.20M revenue,
$2.32M GP (44.6% GM), $1.56M net.
</commit_message>
<xml_diff>
--- a/cfo-dashboard/downloads/cfo-dashboard.xlsx
+++ b/cfo-dashboard/downloads/cfo-dashboard.xlsx
@@ -612,7 +612,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Commercial and Institutional Building Construction (NAICS 236220)  ·  As of 2026-05-07  ·  Source: QuickBooks Online (live, via QuickBooks MCP)</t>
+          <t>Commercial and Institutional Building Construction (NAICS 236220)  ·  As of 2026-07-07  ·  Source: QuickBooks Online (live, via QuickBooks MCP)</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
       <c r="D5" s="5">
         <f>B5-C5</f>
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12736678.98</v>
+        <v>12737250.31</v>
       </c>
       <c r="D6" s="5">
         <f>B6-C6</f>
@@ -703,10 +703,10 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.2718606082616702</v>
+        <v>0.3289685238272541</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.314549467537803</v>
+        <v>0.3145635773804887</v>
       </c>
       <c r="D7" s="6">
         <f>B7-C7</f>
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>9925912.359999999</v>
+        <v>9926483.689999999</v>
       </c>
       <c r="D8" s="5">
         <f>B8-C8</f>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>2810766.62</v>
@@ -775,10 +775,10 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.08575153308354315</v>
+        <v>0.1502665630227206</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.06941567304022843</v>
+        <v>0.06941567305737158</v>
       </c>
       <c r="D10" s="6">
         <f>B10-C10</f>
@@ -1010,29 +1010,29 @@
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Run-rate $46,504,248 vs FY 2025 $40,491,815.</t>
+          <t>Run-rate $51,840,426 vs FY 2025 $40,491,815.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Gross margin compression vs prior year</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>BAD</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Gross margin expansion vs prior year</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>GM% 27.19% vs prior 31.45% (-4.27pt).</t>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>GM% 32.90% vs prior 31.46% (+1.44pt).</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H437"/>
+  <dimension ref="A1:H457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>2026-06-18T00:24:51.804946+00:00</t>
+          <t>2026-07-07T17:35:42.805909+00:00</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
     </row>
     <row r="55">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>14108989.66</v>
+        <v>20292158.47</v>
       </c>
     </row>
     <row r="56">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
     </row>
     <row r="57">
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
     </row>
     <row r="58">
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
     </row>
     <row r="59">
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="B59" s="6" t="n">
-        <v>0.2718606082616702</v>
+        <v>0.3289685238272541</v>
       </c>
     </row>
     <row r="60">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="B60" s="6" t="n">
-        <v>0.08575153308354315</v>
+        <v>0.1502665630227206</v>
       </c>
     </row>
     <row r="61">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B64" s="5" t="n">
-        <v>571765.41</v>
+        <v>997500.28</v>
       </c>
     </row>
     <row r="65">
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="B66" s="5" t="n">
-        <v>16823.83</v>
+        <v>16826.61</v>
       </c>
     </row>
     <row r="67">
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="B68" s="5" t="n">
-        <v>206725</v>
+        <v>396425</v>
       </c>
     </row>
     <row r="69">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B72" s="5" t="n">
-        <v>15924134.62</v>
+        <v>25762267.87</v>
       </c>
     </row>
     <row r="73">
@@ -1959,7 +1959,7 @@
         </is>
       </c>
       <c r="B74" s="5" t="n">
-        <v>2347599</v>
+        <v>2544448.44</v>
       </c>
     </row>
     <row r="75">
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="B76" s="5" t="n">
-        <v>6261029.85</v>
+        <v>8828741.710000001</v>
       </c>
     </row>
     <row r="77">
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="B78" s="5" t="n">
-        <v>2745051.1</v>
+        <v>3895643.04</v>
       </c>
     </row>
     <row r="79">
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="B80" s="5" t="n">
-        <v>529849.5</v>
+        <v>799947.42</v>
       </c>
     </row>
     <row r="81">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B82" s="5" t="n">
-        <v>1928101.09</v>
+        <v>2918142.76</v>
       </c>
     </row>
     <row r="83">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="B84" s="5" t="n">
-        <v>757455.8100000001</v>
+        <v>1109860.58</v>
       </c>
     </row>
     <row r="85">
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="B86" s="5" t="n">
-        <v>72850.52</v>
+        <v>139754.06</v>
       </c>
     </row>
     <row r="87">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="B88" s="5" t="n">
-        <v>191337.16</v>
+        <v>357720.02</v>
       </c>
     </row>
     <row r="89">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="B90" s="5" t="n">
-        <v>64541.24</v>
+        <v>134589.28</v>
       </c>
     </row>
     <row r="91">
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="B92" s="5" t="n">
-        <v>221218.59</v>
+        <v>402320.28</v>
       </c>
     </row>
     <row r="93">
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="B95" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
     </row>
     <row r="96">
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="B96" s="5" t="n">
-        <v>27755136.44</v>
+        <v>27754565.1</v>
       </c>
     </row>
     <row r="97">
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="B97" s="5" t="n">
-        <v>12736678.98</v>
+        <v>12737250.31</v>
       </c>
     </row>
     <row r="98">
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="B98" s="5" t="n">
-        <v>9925912.359999999</v>
+        <v>9926483.689999999</v>
       </c>
     </row>
     <row r="99">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="B100" s="6" t="n">
-        <v>0.314549467537803</v>
+        <v>0.3145635773804887</v>
       </c>
     </row>
     <row r="101">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="B101" s="6" t="n">
-        <v>0.06941567304022843</v>
+        <v>0.06941567305737158</v>
       </c>
     </row>
     <row r="102">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B127" s="5" t="n">
-        <v>33721642.66</v>
+        <v>33721642.65</v>
       </c>
     </row>
     <row r="128">
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="B143" s="5" t="n">
-        <v>1286006.54</v>
+        <v>196030.17</v>
       </c>
     </row>
     <row r="144">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="B151" s="5" t="n">
-        <v>981759.21</v>
+        <v>981248.3100000001</v>
       </c>
     </row>
     <row r="152">
@@ -3493,7 +3493,7 @@
         </is>
       </c>
       <c r="B219" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="220">
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="B220" s="5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="221">
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="B221" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
     </row>
     <row r="222">
@@ -3523,7 +3523,7 @@
         </is>
       </c>
       <c r="B222" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
     </row>
     <row r="223">
@@ -3533,7 +3533,7 @@
         </is>
       </c>
       <c r="B223" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
     </row>
     <row r="224">
@@ -3543,7 +3543,7 @@
         </is>
       </c>
       <c r="B224" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
     </row>
     <row r="225">
@@ -3553,7 +3553,7 @@
         </is>
       </c>
       <c r="B225" s="5" t="n">
-        <v>3875354.04</v>
+        <v>4320035.47</v>
       </c>
     </row>
     <row r="226">
@@ -3563,7 +3563,7 @@
         </is>
       </c>
       <c r="B226" s="5" t="n">
-        <v>1053556.11</v>
+        <v>1421155.69</v>
       </c>
     </row>
     <row r="227">
@@ -3573,7 +3573,7 @@
         </is>
       </c>
       <c r="B227" s="5" t="n">
-        <v>696027.75</v>
+        <v>771998.8100000001</v>
       </c>
     </row>
     <row r="228">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="B228" s="5" t="n">
-        <v>332317.55</v>
+        <v>649156.88</v>
       </c>
     </row>
     <row r="229">
@@ -3593,7 +3593,7 @@
         </is>
       </c>
       <c r="B229" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
     </row>
     <row r="230">
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="B230" s="5" t="n">
-        <v>12642673.27</v>
+        <v>17053868.31</v>
       </c>
     </row>
     <row r="231">
@@ -3613,7 +3613,7 @@
         </is>
       </c>
       <c r="B231" s="5" t="n">
-        <v>8352332.95</v>
+        <v>9263985.720000001</v>
       </c>
     </row>
     <row r="232">
@@ -3623,7 +3623,7 @@
         </is>
       </c>
       <c r="B232" s="5" t="n">
-        <v>3987810.6</v>
+        <v>7789882.59</v>
       </c>
     </row>
     <row r="233">
@@ -3633,7 +3633,7 @@
         </is>
       </c>
       <c r="B233" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
     </row>
     <row r="234">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="B234" s="5" t="n">
-        <v>12642673.27</v>
+        <v>17053868.31</v>
       </c>
     </row>
     <row r="235">
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="B235" s="5" t="n">
-        <v>8352332.95</v>
+        <v>9263985.720000001</v>
       </c>
     </row>
     <row r="236">
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="B236" s="5" t="n">
-        <v>3987810.6</v>
+        <v>7789882.59</v>
       </c>
     </row>
     <row r="237">
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="B237" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
     </row>
     <row r="238">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="B238" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
     </row>
     <row r="239">
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="B239" s="5" t="n">
-        <v>-1103389.81</v>
+        <v>-857832.02</v>
       </c>
     </row>
     <row r="240">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="B240" s="5" t="n">
-        <v>1824082.32</v>
+        <v>1302915.94</v>
       </c>
     </row>
     <row r="241">
@@ -3747,7 +3747,7 @@
         </is>
       </c>
       <c r="B244" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
     </row>
     <row r="245">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="B245" s="13" t="inlineStr">
         <is>
-          <t>YTD avg monthly $3,875,354 continues for 7 months</t>
+          <t>YTD avg monthly $4,320,035 continues for 5 months</t>
         </is>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="B249" s="5" t="n">
-        <v>47158830.4</v>
+        <v>52361634.69</v>
       </c>
     </row>
     <row r="250">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B250" s="13" t="inlineStr">
         <is>
-          <t>Apply prior-year YoY growth +2.4% to remaining 7 months</t>
+          <t>Apply prior-year YoY growth +2.4% to remaining 5 months</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
         </is>
       </c>
       <c r="B251" s="6" t="n">
-        <v>0.02412984854137568</v>
+        <v>0.02412984828845288</v>
       </c>
     </row>
     <row r="252">
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="B255" s="5" t="n">
-        <v>42996995.85</v>
+        <v>47111838.07</v>
       </c>
     </row>
     <row r="256">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B256" s="13" t="inlineStr">
         <is>
-          <t>YTD actual + prior-year avg monthly $3,374,318 × 7 remaining months</t>
+          <t>YTD actual + prior-year avg monthly $3,374,318 × 5 remaining months</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="B260" s="5" t="n">
-        <v>52919774.6</v>
+        <v>67632178.84999999</v>
       </c>
     </row>
     <row r="261">
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="B261" s="5" t="n">
-        <v>44902063.06</v>
+        <v>36770346.65</v>
       </c>
     </row>
     <row r="262">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="B262" s="13" t="inlineStr">
         <is>
-          <t>Avg billings $4,065,858/mo × 7 remaining + YTD; recognized at YTD billings→revenue ratio of 1.18</t>
+          <t>Avg billings $4,065,858/mo × 5 remaining + YTD; recognized at YTD billings→revenue ratio of 1.84</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
         </is>
       </c>
       <c r="B263" s="5" t="n">
-        <v>1.178559981161696</v>
+        <v>1.839313060993898</v>
       </c>
     </row>
     <row r="264">
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="B267" s="5" t="n">
-        <v>47394962.33</v>
+        <v>54736519.32</v>
       </c>
     </row>
     <row r="268">
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="B268" s="5" t="n">
-        <v>42996995.85</v>
+        <v>47111838.07</v>
       </c>
     </row>
     <row r="269">
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="B269" s="5" t="n">
-        <v>52919774.6</v>
+        <v>67632178.84999999</v>
       </c>
     </row>
     <row r="270">
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="B270" s="5" t="n">
-        <v>9922778.75</v>
+        <v>20520340.78</v>
       </c>
     </row>
     <row r="271">
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="B272" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
     </row>
     <row r="273">
@@ -4065,7 +4065,7 @@
         </is>
       </c>
       <c r="B273" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
     </row>
     <row r="274">
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="B274" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
     </row>
     <row r="275">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="B275" s="6" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.1451</v>
       </c>
     </row>
     <row r="276">
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="B277" s="6" t="n">
-        <v>0.0345</v>
+        <v>0.0951</v>
       </c>
     </row>
     <row r="278">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="B280" s="5" t="n">
-        <v>48109881.41</v>
+        <v>56768366.09</v>
       </c>
     </row>
     <row r="281">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="B281" s="5" t="n">
-        <v>12116983.99</v>
+        <v>17539638.27</v>
       </c>
     </row>
     <row r="282">
@@ -4157,7 +4157,7 @@
         </is>
       </c>
       <c r="B282" s="6" t="n">
-        <v>0.2518606081952797</v>
+        <v>0.3089685237536482</v>
       </c>
     </row>
     <row r="283">
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="B283" s="5" t="n">
-        <v>3451957.75</v>
+        <v>7735630.13</v>
       </c>
     </row>
     <row r="284">
@@ -4177,7 +4177,7 @@
         </is>
       </c>
       <c r="B284" s="6" t="n">
-        <v>0.07175153307616747</v>
+        <v>0.1362665629441902</v>
       </c>
     </row>
     <row r="285">
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="B286" s="5" t="n">
-        <v>49770951.38</v>
+        <v>62164755.51</v>
       </c>
     </row>
     <row r="287">
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="B287" s="5" t="n">
-        <v>11539923.06</v>
+        <v>17963657.63</v>
       </c>
     </row>
     <row r="288">
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="B288" s="6" t="n">
-        <v>0.2318606081952797</v>
+        <v>0.2889685237536482</v>
       </c>
     </row>
     <row r="289">
@@ -4227,7 +4227,7 @@
         </is>
       </c>
       <c r="B289" s="5" t="n">
-        <v>2874348.75</v>
+        <v>7600670.99</v>
       </c>
     </row>
     <row r="290">
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="B290" s="6" t="n">
-        <v>0.05775153307616747</v>
+        <v>0.1222665629441902</v>
       </c>
     </row>
     <row r="291">
@@ -4259,7 +4259,7 @@
         </is>
       </c>
       <c r="B292" s="6" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.1451</v>
       </c>
     </row>
     <row r="293">
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="B295" s="5" t="n">
-        <v>50435093.83</v>
+        <v>59360387.37</v>
       </c>
     </row>
     <row r="296">
@@ -4299,7 +4299,7 @@
         </is>
       </c>
       <c r="B296" s="5" t="n">
-        <v>13711315.28</v>
+        <v>19527699</v>
       </c>
     </row>
     <row r="297">
@@ -4309,7 +4309,7 @@
         </is>
       </c>
       <c r="B297" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
     </row>
     <row r="298">
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="B298" s="5" t="n">
-        <v>4324886.62</v>
+        <v>8919881.390000001</v>
       </c>
     </row>
     <row r="299">
@@ -4329,7 +4329,7 @@
         </is>
       </c>
       <c r="B299" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
     </row>
     <row r="300">
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="B301" s="5" t="n">
-        <v>54698200.15</v>
+        <v>67971193.18000001</v>
       </c>
     </row>
     <row r="302">
@@ -4359,7 +4359,7 @@
         </is>
       </c>
       <c r="B302" s="5" t="n">
-        <v>14870285.96</v>
+        <v>22360383.08</v>
       </c>
     </row>
     <row r="303">
@@ -4369,7 +4369,7 @@
         </is>
       </c>
       <c r="B303" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
     </row>
     <row r="304">
@@ -4379,7 +4379,7 @@
         </is>
       </c>
       <c r="B304" s="5" t="n">
-        <v>4690454.52</v>
+        <v>10213797.58</v>
       </c>
     </row>
     <row r="305">
@@ -4389,7 +4389,7 @@
         </is>
       </c>
       <c r="B305" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
     </row>
     <row r="306">
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="B307" s="6" t="n">
-        <v>0.1245</v>
+        <v>0.1851</v>
       </c>
     </row>
     <row r="308">
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="B310" s="5" t="n">
-        <v>52295263.77</v>
+        <v>61434004.4</v>
       </c>
     </row>
     <row r="311">
@@ -4451,7 +4451,7 @@
         </is>
       </c>
       <c r="B311" s="5" t="n">
-        <v>15001451.17</v>
+        <v>21131363.8</v>
       </c>
     </row>
     <row r="312">
@@ -4461,7 +4461,7 @@
         </is>
       </c>
       <c r="B312" s="6" t="n">
-        <v>0.2868606081952797</v>
+        <v>0.3439685237536482</v>
       </c>
     </row>
     <row r="313">
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="B313" s="5" t="n">
-        <v>5033499.31</v>
+        <v>9876533.74</v>
       </c>
     </row>
     <row r="314">
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="B314" s="6" t="n">
-        <v>0.09625153307616746</v>
+        <v>0.1607665629441902</v>
       </c>
     </row>
     <row r="315">
@@ -4501,7 +4501,7 @@
         </is>
       </c>
       <c r="B316" s="5" t="n">
-        <v>58807414.45</v>
+        <v>72802968.84999999</v>
       </c>
     </row>
     <row r="317">
@@ -4511,7 +4511,7 @@
         </is>
       </c>
       <c r="B317" s="5" t="n">
-        <v>17751641.89</v>
+        <v>26133974.25</v>
       </c>
     </row>
     <row r="318">
@@ -4521,7 +4521,7 @@
         </is>
       </c>
       <c r="B318" s="6" t="n">
-        <v>0.3018606081952797</v>
+        <v>0.3589685237536482</v>
       </c>
     </row>
     <row r="319">
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="B319" s="5" t="n">
-        <v>6277781.65</v>
+        <v>12468714.25</v>
       </c>
     </row>
     <row r="320">
@@ -4541,7 +4541,7 @@
         </is>
       </c>
       <c r="B320" s="6" t="n">
-        <v>0.1067515330761675</v>
+        <v>0.1712665629441902</v>
       </c>
     </row>
     <row r="321">
@@ -5629,166 +5629,378 @@
     <row r="423">
       <c r="A423" s="29" t="inlineStr">
         <is>
-          <t>benchmark.companyName</t>
+          <t>verifiedMonths[4].periodStart</t>
         </is>
       </c>
       <c r="B423" s="13" t="inlineStr">
         <is>
-          <t>Midwest Design Group LLC</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="29" t="inlineStr">
         <is>
-          <t>benchmark.metricType</t>
+          <t>verifiedMonths[4].periodEnd</t>
         </is>
       </c>
       <c r="B424" s="13" t="inlineStr">
         <is>
-          <t>profit</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="29" t="inlineStr">
         <is>
-          <t>benchmark.metricLabel</t>
-        </is>
-      </c>
-      <c r="B425" s="13" t="inlineStr">
-        <is>
-          <t>Yearly Profit</t>
-        </is>
+          <t>verifiedMonths[4].revenue</t>
+        </is>
+      </c>
+      <c r="B425" s="5" t="n">
+        <v>4925779.55</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="29" t="inlineStr">
         <is>
-          <t>benchmark.metricValue</t>
+          <t>verifiedMonths[4].cogs</t>
         </is>
       </c>
       <c r="B426" s="5" t="n">
-        <v>3757685.49</v>
+        <v>3335298.81</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="29" t="inlineStr">
         <is>
-          <t>benchmark.regionalAverage</t>
+          <t>verifiedMonths[4].grossProfit</t>
         </is>
       </c>
       <c r="B427" s="5" t="n">
-        <v>101486.51</v>
+        <v>1590480.74</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="29" t="inlineStr">
         <is>
-          <t>benchmark.nationalAverage</t>
-        </is>
-      </c>
-      <c r="B428" s="13" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>verifiedMonths[4].operatingExpenses</t>
+        </is>
+      </c>
+      <c r="B428" s="5" t="n">
+        <v>978876.21</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="29" t="inlineStr">
         <is>
-          <t>benchmark.vsRegionalPercent</t>
+          <t>verifiedMonths[4].netIncome</t>
         </is>
       </c>
       <c r="B429" s="5" t="n">
-        <v>3602.65</v>
+        <v>611696.3100000001</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="29" t="inlineStr">
         <is>
-          <t>benchmark.vsNationalPercent</t>
+          <t>verifiedMonths[4].grossMarginPct</t>
         </is>
       </c>
       <c r="B430" s="6" t="n">
-        <v>0</v>
+        <v>0.3228891435062294</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="29" t="inlineStr">
         <is>
-          <t>benchmark.isAboveRegional</t>
-        </is>
-      </c>
-      <c r="B431" s="6" t="b">
-        <v>1</v>
+          <t>verifiedMonths[4].netMarginPct</t>
+        </is>
+      </c>
+      <c r="B431" s="6" t="n">
+        <v>0.1241826402888859</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="29" t="inlineStr">
         <is>
-          <t>benchmark.isAboveNational</t>
-        </is>
-      </c>
-      <c r="B432" s="6" t="b">
-        <v>0</v>
+          <t>verifiedMonths[4].month</t>
+        </is>
+      </c>
+      <c r="B432" s="13" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="29" t="inlineStr">
         <is>
-          <t>benchmark.location</t>
+          <t>verifiedMonths[5].periodStart</t>
         </is>
       </c>
       <c r="B433" s="13" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="29" t="inlineStr">
         <is>
-          <t>benchmark.naicsCode</t>
+          <t>verifiedMonths[5].periodEnd</t>
         </is>
       </c>
       <c r="B434" s="13" t="inlineStr">
         <is>
-          <t>236220</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="29" t="inlineStr">
         <is>
-          <t>benchmark.industryType</t>
-        </is>
-      </c>
-      <c r="B435" s="13" t="inlineStr">
-        <is>
-          <t>Commercial And Institutional Building Construction</t>
-        </is>
+          <t>verifiedMonths[5].revenue</t>
+        </is>
+      </c>
+      <c r="B435" s="5" t="n">
+        <v>5199082.25</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="29" t="inlineStr">
         <is>
-          <t>benchmark.benchmarkPeriodRange</t>
-        </is>
-      </c>
-      <c r="B436" s="13" t="inlineStr">
-        <is>
-          <t>Mar 2025 - Feb 2026</t>
-        </is>
+          <t>verifiedMonths[5].cogs</t>
+        </is>
+      </c>
+      <c r="B436" s="5" t="n">
+        <v>2879916.44</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="29" t="inlineStr">
         <is>
+          <t>verifiedMonths[5].grossProfit</t>
+        </is>
+      </c>
+      <c r="B437" s="5" t="n">
+        <v>2319165.81</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="29" t="inlineStr">
+        <is>
+          <t>verifiedMonths[5].operatingExpenses</t>
+        </is>
+      </c>
+      <c r="B438" s="5" t="n">
+        <v>757595.17</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="29" t="inlineStr">
+        <is>
+          <t>verifiedMonths[5].netIncome</t>
+        </is>
+      </c>
+      <c r="B439" s="5" t="n">
+        <v>1561681.96</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="29" t="inlineStr">
+        <is>
+          <t>verifiedMonths[5].grossMarginPct</t>
+        </is>
+      </c>
+      <c r="B440" s="6" t="n">
+        <v>0.4460721524457514</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="29" t="inlineStr">
+        <is>
+          <t>verifiedMonths[5].netMarginPct</t>
+        </is>
+      </c>
+      <c r="B441" s="6" t="n">
+        <v>0.3003764674044155</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="29" t="inlineStr">
+        <is>
+          <t>verifiedMonths[5].month</t>
+        </is>
+      </c>
+      <c r="B442" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.companyName</t>
+        </is>
+      </c>
+      <c r="B443" s="13" t="inlineStr">
+        <is>
+          <t>Midwest Design Group LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.metricType</t>
+        </is>
+      </c>
+      <c r="B444" s="13" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.metricLabel</t>
+        </is>
+      </c>
+      <c r="B445" s="13" t="inlineStr">
+        <is>
+          <t>Yearly Profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.metricValue</t>
+        </is>
+      </c>
+      <c r="B446" s="5" t="n">
+        <v>3757685.49</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.regionalAverage</t>
+        </is>
+      </c>
+      <c r="B447" s="5" t="n">
+        <v>101486.51</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.nationalAverage</t>
+        </is>
+      </c>
+      <c r="B448" s="13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.vsRegionalPercent</t>
+        </is>
+      </c>
+      <c r="B449" s="5" t="n">
+        <v>3602.65</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.vsNationalPercent</t>
+        </is>
+      </c>
+      <c r="B450" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.isAboveRegional</t>
+        </is>
+      </c>
+      <c r="B451" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.isAboveNational</t>
+        </is>
+      </c>
+      <c r="B452" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.location</t>
+        </is>
+      </c>
+      <c r="B453" s="13" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.naicsCode</t>
+        </is>
+      </c>
+      <c r="B454" s="13" t="inlineStr">
+        <is>
+          <t>236220</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.industryType</t>
+        </is>
+      </c>
+      <c r="B455" s="13" t="inlineStr">
+        <is>
+          <t>Commercial And Institutional Building Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="29" t="inlineStr">
+        <is>
+          <t>benchmark.benchmarkPeriodRange</t>
+        </is>
+      </c>
+      <c r="B456" s="13" t="inlineStr">
+        <is>
+          <t>Mar 2025 - Feb 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="29" t="inlineStr">
+        <is>
           <t>benchmark.reportDate</t>
         </is>
       </c>
-      <c r="B437" s="13" t="inlineStr">
+      <c r="B457" s="13" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
@@ -5829,7 +6041,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>YTD 2026 (2026-01-01 → 2026-05-07) vs FY 2025</t>
+          <t>YTD 2026 (2026-01-01 → 2026-07-07) vs FY 2025</t>
         </is>
       </c>
     </row>
@@ -5867,10 +6079,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
       <c r="D5" s="5">
         <f>B5-C5</f>
@@ -5888,10 +6100,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>14108989.66</v>
+        <v>20292158.47</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>27755136.44</v>
+        <v>27754565.1</v>
       </c>
       <c r="D6" s="5">
         <f>B6-C6</f>
@@ -5952,10 +6164,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>9925912.359999999</v>
+        <v>9926483.689999999</v>
       </c>
       <c r="D9" s="5">
         <f>B9-C9</f>
@@ -6032,7 +6244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6096,10 +6308,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>39537774.9</v>
@@ -6120,10 +6332,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12736678.98</v>
+        <v>12737250.31</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>11102557.97</v>
@@ -6144,10 +6356,10 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.2718606082616702</v>
+        <v>0.3289685238272541</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.314549467537803</v>
+        <v>0.3145635773804887</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0.2808088719732179</v>
@@ -6164,10 +6376,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>9925912.359999999</v>
+        <v>9926483.689999999</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>8249044.14</v>
@@ -6188,7 +6400,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>2810766.62</v>
@@ -6212,10 +6424,10 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.08575153308354315</v>
+        <v>0.1502665630227206</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.06941567304022843</v>
+        <v>0.06941567305737158</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>0.07332639652415061</v>
@@ -6399,6 +6611,70 @@
       </c>
       <c r="H18" s="6">
         <f>IFERROR(G18/B18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4925779.55</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>3335298.81</v>
+      </c>
+      <c r="D19" s="5">
+        <f>B19-C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="6">
+        <f>IFERROR(D19/B19,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>978876.21</v>
+      </c>
+      <c r="G19" s="5">
+        <f>D19-F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="6">
+        <f>IFERROR(G19/B19,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>5199082.25</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>2879916.44</v>
+      </c>
+      <c r="D20" s="5">
+        <f>B20-C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
+        <f>IFERROR(D20/B20,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>757595.17</v>
+      </c>
+      <c r="G20" s="5">
+        <f>D20-F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="6">
+        <f>IFERROR(G20/B20,0)</f>
         <v/>
       </c>
     </row>
@@ -6469,10 +6745,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
       <c r="D6" s="5">
         <f>B6-C6</f>
@@ -6486,10 +6762,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>14108989.66</v>
+        <v>20292158.47</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>27755136.44</v>
+        <v>27754565.1</v>
       </c>
       <c r="D7" s="5">
         <f>B7-C7</f>
@@ -6503,10 +6779,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>12736678.98</v>
+        <v>12737250.31</v>
       </c>
       <c r="D8" s="5">
         <f>B8-C8</f>
@@ -6520,10 +6796,10 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.2718606082616702</v>
+        <v>0.3289685238272541</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.314549467537803</v>
+        <v>0.3145635773804887</v>
       </c>
       <c r="D9" s="6">
         <f>B9-C9</f>
@@ -6537,10 +6813,10 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>9925912.359999999</v>
+        <v>9926483.689999999</v>
       </c>
       <c r="D10" s="5">
         <f>B10-C10</f>
@@ -6554,7 +6830,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>2810766.62</v>
@@ -6733,7 +7009,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5 of 12 months completed · 7 remaining. Year-End Forecast = YTD + (Avg Monthly × Remaining).</t>
+          <t>7 of 12 months completed · 5 remaining. Year-End Forecast = YTD + (Avg Monthly × Remaining).</t>
         </is>
       </c>
     </row>
@@ -6771,13 +7047,13 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>3875354.04</v>
+        <v>4320035.47</v>
       </c>
       <c r="D5" s="5">
-        <f>B5+C5*7</f>
+        <f>B5+C5*5</f>
         <v/>
       </c>
       <c r="E5" s="5">
@@ -6792,13 +7068,13 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1053556.11</v>
+        <v>1421155.69</v>
       </c>
       <c r="D6" s="5">
-        <f>B6+C6*7</f>
+        <f>B6+C6*5</f>
         <v/>
       </c>
       <c r="E6" s="5">
@@ -6813,13 +7089,13 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3480138.73</v>
+        <v>5403991.67</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>696027.75</v>
+        <v>771998.8100000001</v>
       </c>
       <c r="D7" s="5">
-        <f>B7+C7*7</f>
+        <f>B7+C7*5</f>
         <v/>
       </c>
       <c r="E7" s="5">
@@ -6834,13 +7110,13 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>332317.55</v>
+        <v>649156.88</v>
       </c>
       <c r="D8" s="5">
-        <f>B8+C8*7</f>
+        <f>B8+C8*5</f>
         <v/>
       </c>
       <c r="E8" s="5">
@@ -6877,7 +7153,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>-1103389.81</v>
+        <v>-857832.02</v>
       </c>
     </row>
   </sheetData>
@@ -6895,7 +7171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6983,19 +7259,19 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>40491815.42</v>
+        <v>40491815.41</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>12736678.98</v>
+        <v>12737250.31</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.314549467537803</v>
+        <v>0.3145635773804887</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>2810766.62</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.06941567304022843</v>
+        <v>0.06941567305737158</v>
       </c>
     </row>
     <row r="7">
@@ -7005,19 +7281,19 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>5267780.53</v>
+        <v>9948089.85</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.2718606082616702</v>
+        <v>0.3289685238272541</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1661587.75</v>
+        <v>4544098.18</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.08575153308354315</v>
+        <v>0.1502665630227206</v>
       </c>
     </row>
     <row r="8">
@@ -7027,19 +7303,19 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>12642673.27</v>
+        <v>17053868.31</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>3987810.6</v>
+        <v>7789882.59</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
     </row>
     <row r="11">
@@ -7201,6 +7477,62 @@
       </c>
       <c r="H16" s="6" t="n">
         <v>0.1474627544988424</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4925779.55</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>3335298.81</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1590480.74</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>978876.21</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>611696.3100000001</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>0.3228891435062294</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0.1241826402888859</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5199082.25</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>2879916.44</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>2319165.81</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>757595.17</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>1561681.96</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>0.4460721524457514</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0.3003764674044155</v>
       </c>
     </row>
   </sheetData>
@@ -7281,7 +7613,7 @@
         <v>20720.33</v>
       </c>
       <c r="C6" s="6">
-        <f>B6/19376770.19</f>
+        <f>B6/30240248.32</f>
         <v/>
       </c>
       <c r="D6" s="5" t="n">
@@ -7295,10 +7627,10 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>571765.41</v>
+        <v>997500.28</v>
       </c>
       <c r="C7" s="6">
-        <f>B7/19376770.19</f>
+        <f>B7/30240248.32</f>
         <v/>
       </c>
       <c r="D7" s="5" t="n">
@@ -7312,10 +7644,10 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>16823.83</v>
+        <v>16826.61</v>
       </c>
       <c r="C8" s="6">
-        <f>B8/19376770.19</f>
+        <f>B8/30240248.32</f>
         <v/>
       </c>
       <c r="D8" s="5" t="n">
@@ -7329,10 +7661,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>206725</v>
+        <v>396425</v>
       </c>
       <c r="C9" s="6">
-        <f>B9/19376770.19</f>
+        <f>B9/30240248.32</f>
         <v/>
       </c>
       <c r="D9" s="5" t="n">
@@ -7349,7 +7681,7 @@
         <v>4820</v>
       </c>
       <c r="C10" s="6">
-        <f>B10/19376770.19</f>
+        <f>B10/30240248.32</f>
         <v/>
       </c>
       <c r="D10" s="5" t="n">
@@ -7363,14 +7695,14 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>15924134.62</v>
+        <v>25762267.87</v>
       </c>
       <c r="C11" s="6">
-        <f>B11/19376770.19</f>
+        <f>B11/30240248.32</f>
         <v/>
       </c>
       <c r="D11" s="5" t="n">
-        <v>33721642.66</v>
+        <v>33721642.65</v>
       </c>
     </row>
     <row r="12">
@@ -7380,10 +7712,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>2347599</v>
+        <v>2544448.44</v>
       </c>
       <c r="C12" s="6">
-        <f>B12/19376770.19</f>
+        <f>B12/30240248.32</f>
         <v/>
       </c>
       <c r="D12" s="5" t="n">
@@ -7426,10 +7758,10 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>6261029.85</v>
+        <v>8828741.710000001</v>
       </c>
       <c r="C17" s="6">
-        <f>B17/14108989.66</f>
+        <f>B17/20292158.47</f>
         <v/>
       </c>
       <c r="D17" s="5" t="n">
@@ -7443,10 +7775,10 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2745051.1</v>
+        <v>3895643.04</v>
       </c>
       <c r="C18" s="6">
-        <f>B18/14108989.66</f>
+        <f>B18/20292158.47</f>
         <v/>
       </c>
       <c r="D18" s="5" t="n">
@@ -7460,10 +7792,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>529849.5</v>
+        <v>799947.42</v>
       </c>
       <c r="C19" s="6">
-        <f>B19/14108989.66</f>
+        <f>B19/20292158.47</f>
         <v/>
       </c>
       <c r="D19" s="5" t="n">
@@ -7511,10 +7843,10 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1928101.09</v>
+        <v>2918142.76</v>
       </c>
       <c r="C24" s="6">
-        <f>B24/3480138.73</f>
+        <f>B24/5403991.67</f>
         <v/>
       </c>
       <c r="D24" s="5" t="n">
@@ -7532,14 +7864,14 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>757455.8100000001</v>
+        <v>1109860.58</v>
       </c>
       <c r="C25" s="6">
-        <f>B25/3480138.73</f>
+        <f>B25/5403991.67</f>
         <v/>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1286006.54</v>
+        <v>196030.17</v>
       </c>
       <c r="E25" s="6">
         <f>IFERROR((B25-D25)/ABS(D25),"")</f>
@@ -7553,10 +7885,10 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>72850.52</v>
+        <v>139754.06</v>
       </c>
       <c r="C26" s="6">
-        <f>B26/3480138.73</f>
+        <f>B26/5403991.67</f>
         <v/>
       </c>
       <c r="D26" s="5" t="n">
@@ -7574,10 +7906,10 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>191337.16</v>
+        <v>357720.02</v>
       </c>
       <c r="C27" s="6">
-        <f>B27/3480138.73</f>
+        <f>B27/5403991.67</f>
         <v/>
       </c>
       <c r="D27" s="5" t="n">
@@ -7595,10 +7927,10 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>64541.24</v>
+        <v>134589.28</v>
       </c>
       <c r="C28" s="6">
-        <f>B28/3480138.73</f>
+        <f>B28/5403991.67</f>
         <v/>
       </c>
       <c r="D28" s="5" t="n">
@@ -7616,14 +7948,14 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>221218.59</v>
+        <v>402320.28</v>
       </c>
       <c r="C29" s="6">
-        <f>B29/3480138.73</f>
+        <f>B29/5403991.67</f>
         <v/>
       </c>
       <c r="D29" s="5" t="n">
-        <v>981759.21</v>
+        <v>981248.3100000001</v>
       </c>
       <c r="E29" s="6">
         <f>IFERROR((B29-D29)/ABS(D29),"")</f>
@@ -7917,7 +8249,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>19376770.19</v>
+        <v>30240248.32</v>
       </c>
     </row>
     <row r="6">
@@ -7986,10 +8318,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>46504248.46</v>
+        <v>51840425.69</v>
       </c>
       <c r="C12" s="5">
-        <f>B5+(3875354.04*7)*(1+$B$6)</f>
+        <f>B5+(4320035.47*5)*(1+$B$6)</f>
         <v/>
       </c>
       <c r="D12" s="5">
@@ -8004,10 +8336,10 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.2718606081952797</v>
+        <v>0.3289685237536482</v>
       </c>
       <c r="C13" s="6">
-        <f>0.2718606081952797+$B$7</f>
+        <f>0.3289685237536482+$B$7</f>
         <v/>
       </c>
       <c r="D13" s="6">
@@ -8022,7 +8354,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>12642673.27</v>
+        <v>17053868.31</v>
       </c>
       <c r="C14" s="5">
         <f>C12*C13</f>
@@ -8040,10 +8372,10 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>8352332.95</v>
+        <v>9263985.720000001</v>
       </c>
       <c r="C15" s="5">
-        <f>3480138.73+(696027.75*7)*(1+$B$8)</f>
+        <f>5403991.67+(771998.81*5)*(1+$B$8)</f>
         <v/>
       </c>
       <c r="D15" s="5">
@@ -8058,7 +8390,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>3987810.6</v>
+        <v>7789882.59</v>
       </c>
       <c r="C16" s="5">
         <f>C14-C15</f>
@@ -8076,7 +8408,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.08575153307616747</v>
+        <v>0.1502665629441902</v>
       </c>
       <c r="C17" s="6">
         <f>C16/C12</f>

</xml_diff>